<commit_message>
Apply management decisions: owner, Texas 3-year rule, forfeiture clauses, revenue timing
Director of Financial Reporting and Analysis replaces the Controller as owner
of the quarterly review and annual filings. Texas 3-year rule adopted; the
1-year wage rule is not applied. Philly and TUR forfeiture clauses are not
relied on against an escheat claim. Fee checks stay in the ordinary matching
process and the year-end revenue true-up; only amounts written off at a
quarterly review are booked to revenue. Added the after-remittance process
(holder relief and reimbursement sections verified for all five states) and
a rollout note tab on the briefing doc. Workbook rebuilt; Summary still ties
to 226,764.46 with no figure change.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SVpE7ymJvQuwNuD1Yq5LvD
</commit_message>
<xml_diff>
--- a/accrued-commissions-analysis/Accrued_Commissions_Unclaimed_Property_Analysis.xlsx
+++ b/accrued-commissions-analysis/Accrued_Commissions_Unclaimed_Property_Analysis.xlsx
@@ -111,7 +111,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1684" uniqueCount="736">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1693" uniqueCount="744">
   <si>
     <t xml:space="preserve">Accrued Commissions - Unclaimed Property Exposure by Entity</t>
   </si>
@@ -206,13 +206,13 @@
     <t xml:space="preserve">Dormant at next report cutoff - LONG - likely-commission + memo-flagged</t>
   </si>
   <si>
-    <t xml:space="preserve">Likely test given independent-contractor agents</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dormant today - LIKELY test - likely-commission + memo-flagged</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dormant at next report cutoff - LIKELY test - likely-commission + memo-flagged</t>
+    <t xml:space="preserve">Adopted test given independent-contractor agents</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dormant today - ADOPTED test - likely-commission + memo-flagged</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dormant at next report cutoff - ADOPTED test - likely-commission + memo-flagged</t>
   </si>
   <si>
     <t xml:space="preserve">Oldest item</t>
@@ -293,13 +293,13 @@
     <t xml:space="preserve">How to read this</t>
   </si>
   <si>
-    <t xml:space="preserve">Classification (Detail col N) uses the fee amounts in rows 4-7 and the threshold in B8: an exact fee amount = presumed company revenue (keep; book to revenue, not unclaimed property). At or under the threshold = likely fee, review. Memo-flagged = memo says not ours / unknown agent / duplicate / legal hold (owed back to the payer or needs resolution). Everything else = larger amount that likely includes an agent's commission split - this is the unclaimed-property population.</t>
+    <t xml:space="preserve">Classification (Detail col N) uses the fee amounts in rows 4-7 and the threshold in B8: an exact fee amount = company revenue, not unclaimed property. Decision 10/6/2026: fee checks are NOT moved to revenue en masse; they are recognized through the ordinary matching process and the year-end revenue true-up, and only an item being written off at a quarterly threshold review is booked to revenue at that time. At or under the threshold = likely fee, review. Memo-flagged = memo says not ours / unknown agent / duplicate / legal hold (owed back to the payer or needs resolution). Everything else = larger amount that likely includes an agent's commission split - this is the unclaimed-property population.</t>
   </si>
   <si>
     <t xml:space="preserve">Columns R-S apply the dormancy tests to ALL unbooked items (upper bound). Columns T-W apply them only to the likely-commission and memo-flagged items. Even the T-W figures are upper bounds: within a larger check, only the agent's share (typically the check less the company's fee / split) is reportable; the company's share is revenue.</t>
   </si>
   <si>
-    <t xml:space="preserve">SHORT test = the state's period for wages / compensation for personal services. LONG test = the general catch-all period. Column X picks the likely test for each entity's default governing state now that agents are confirmed to be independent contractors (Texas and Florida: LONG; Illinois, Pennsylvania, Alabama: SHORT), and columns Y-Z apply it item by item, so an item whose owner state has been filled in uses its own state's test. See State Rules cols M-N for the reasoning; it is a legal judgment for counsel to confirm.</t>
+    <t xml:space="preserve">SHORT test = the state's period for wages / compensation for personal services. LONG test = the general catch-all period. Column X picks the likely test for each entity's default governing state now that agents are confirmed to be independent contractors (Texas and Florida: LONG; Illinois, Pennsylvania, Alabama: SHORT), and columns Y-Z apply it item by item, so an item whose owner state has been filled in uses its own state's test. See State Rules cols M-N for the basis. Management adopted these tests on 10/6/2026 after the statutes were verified; Texas applies the 3-year rule and the 1-year wage rule is not used.</t>
   </si>
   <si>
     <t xml:space="preserve">Unknown agent = second priority rule. Per the Entity Management Database, URE Dallas, URE Houston, Quick Close Properties (TUR), URE Chicago and URE Philadelphia are all TEXAS LLCs; Gallery (RaySon Partners) is Florida; Leading Edge Realty is Alabama. Column B holds that formation state as each entity's DEFAULT governing state, so unknown-agent items at Chicago and Philly are tested under TEXAS rules (3-year general period for contractor commissions), not Illinois or Pennsylvania. When an agent's last-known address state is entered in Detail col U, that item switches to the address state's rules (first priority rule). Office state is shown in col AB for reference.</t>
@@ -398,13 +398,13 @@
     <t xml:space="preserve">Heuristic reportable population $ (larger-amount + memo-flagged items)</t>
   </si>
   <si>
-    <t xml:space="preserve">Likely test for this item's governing state</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dormant date - LIKELY test</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dormant at next cutoff - LIKELY test?</t>
+    <t xml:space="preserve">Adopted test for this item's governing state</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dormant date - ADOPTED test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dormant at next cutoff - ADOPTED test?</t>
   </si>
   <si>
     <t xml:space="preserve">1839</t>
@@ -1685,7 +1685,7 @@
     <t xml:space="preserve">ICA CLAUSES THAT REDUCE WHAT IS OWED TO AGENTS - legal question</t>
   </si>
   <si>
-    <t xml:space="preserve">Every ICA lets the Broker hold or apply commissions against amounts the agent owes (dues, fees, E&amp;O deductibles, indemnity) and conditions post-termination payouts on dues being paid in full. The Philly ICA goes further: an incomplete file 30 days past closing is paid 50/50 and 60 days past closing is 'forfeited'; a license not reactivated within 30 days means 'brokerage will keep 100% of commission'. TUR's agreement forfeits accrued commissions if the agent collects in their own name or breaches Section 5. A documented offset reduces the agent's share dollar for dollar. A contractual forfeiture is less certain. Verified 10/6/2026: Texas (Prop. Code 74.308), Illinois (765 ILCS 1026/15-610(a)), Florida (717.129(1)) and Alabama (35-12-88(a)) each say that the expiration of a period specified by CONTRACT does not prevent property from being presumed abandoned, and Texas 74.309 separately bars taking funds into income by private agreement to circumvent the unclaimed property process. Pennsylvania's 1301.16 mentions only statute and court order, not contract, and has no private-escheat section, so the Philly clause is a contract-law question there; but most Philly items default to Texas, where 74.308-74.309 apply. Whether any state would honor these clauses against an escheat claim is for counsel. Do not treat a forfeiture as the company's money until counsel says so AND the triggering facts (closing date, file status at day 60, termination date) are documented per item. See the ICA Terms tab.</t>
+    <t xml:space="preserve">Every ICA lets the Broker hold or apply commissions against amounts the agent owes (dues, fees, E&amp;O deductibles, indemnity) and conditions post-termination payouts on dues being paid in full. The Philly ICA goes further: an incomplete file 30 days past closing is paid 50/50 and 60 days past closing is 'forfeited'; a license not reactivated within 30 days means 'brokerage will keep 100% of commission'. TUR's agreement forfeits accrued commissions if the agent collects in their own name or breaches Section 5. A documented offset reduces the agent's share dollar for dollar. A contractual forfeiture is less certain. Verified 10/6/2026: Texas (Prop. Code 74.308), Illinois (765 ILCS 1026/15-610(a)), Florida (717.129(1)) and Alabama (35-12-88(a)) each say that the expiration of a period specified by CONTRACT does not prevent property from being presumed abandoned, and Texas 74.309 separately bars taking funds into income by private agreement to circumvent the unclaimed property process. Pennsylvania's 1301.16 mentions only statute and court order, not contract, and has no private-escheat section, so the Philly clause is a contract-law question there; but most Philly items default to Texas, where 74.308-74.309 apply. DECISION 10/6/2026: the company does not rely on the forfeiture clauses against an escheat claim. An item past dormancy is paid or reported at the agent's share regardless of the Philly 60-day / license clauses or the TUR breach clauses. Documented offsets still reduce the agent's share dollar for dollar. See the ICA Terms tab.</t>
   </si>
   <si>
     <t xml:space="preserve">Counsel; Accounting to document per item.</t>
@@ -1760,10 +1760,34 @@
     <t xml:space="preserve">Counsel.</t>
   </si>
   <si>
+    <t xml:space="preserve">DECISION: revenue timing for fee checks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fee checks and confirmed small items are company revenue and are not unclaimed property, but they are NOT moved to revenue en masse. They stay in the accrued balance and are recognized when matched in the ordinary course and through the year-end revenue true-up, which already captures them. At a quarterly threshold review only an item that is being written off at that time is booked to revenue (decision 10/6/2026).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Director of Financial Reporting and Analysis.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DECISION: process owner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The quarterly threshold review and the annual state filings are owned by the Director of Financial Reporting and Analysis, with counsel; the CFO approves any VDA and any retention under an offset (decision 10/6/2026).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AFTER REMITTANCE: the agent later submits the file</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Good-faith delivery to the state relieves the holder of liability for the property in every state in scope (Tex. Prop. Code 74.304(b)-(c); 72 P.S. 1301.14; Fla. Stat. 717.1201(1); Ala. Code 35-12-79(b); 765 ILCS 1026/15-604). The transaction is still processed and the agent is still paid: either the agent claims the money from the state, or the company pays the agent and files for reimbursement from the state (Texas 74.502: the Comptroller reimburses a valid claim paid by the holder; Pennsylvania 1301.14: reimbursement with interest; Florida 717.1201(3); Alabama 35-12-79(c); Illinois 15-605). The company's fee on that transaction is revenue as usual. Keep the state report reference on the Paperless Pipeline transaction so the reimbursement claim can be filed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Director of Financial Reporting and Analysis / Accounting.</t>
+  </si>
+  <si>
     <t xml:space="preserve">VERIFIED 10/6/2026 - and what is still open</t>
   </si>
   <si>
-    <t xml:space="preserve">Every rule on the State Rules tab for TX, IL, PA, FL and AL (periods, section numbers, report cutoff and due date, due-diligence threshold and timing, VDA terms, anti-limitation provision) was read from the statute text and the state treasury pages on 10/6/2026; the URLs are in the Sources column. Corrections made: IL business holders file by May 1 for the calendar year (not November 1 / June 30); FL's operative long period for a Florida holder with an unknown owner address is 3 years under 717.1035 (not 5); the PA commissions rule is 1301.10(2) (not 1301.5); PA, FL and TX VDA descriptions replaced with the treasury pages' own terms. STILL OPEN: (1) no court decision or Comptroller ruling specifically on broker-to-agent commissions was found - the Texas 3-year position rests on the statutory definitions and the Comptroller's MS02 table; (2) whether a court would enforce the Philly ICA 60-day forfeiture against an escheat claim (the PA statute is silent on contract-based bars; TX 74.308-74.309 cut against it); (3) deposit date is a proxy for the payable date; (4) Missouri and DC not researched (no holder formed there, DC balance $0); (5) Texas VDA eligibility for an entity that has filed before is not stated on the Comptroller pages - ask when requesting.</t>
+    <t xml:space="preserve">Every rule on the State Rules tab for TX, IL, PA, FL and AL (periods, section numbers, report cutoff and due date, due-diligence threshold and timing, VDA terms, anti-limitation provision) was read from the statute text and the state treasury pages on 10/6/2026; the URLs are in the Sources column. Corrections made: IL business holders file by May 1 for the calendar year (not November 1 / June 30); FL's operative long period for a Florida holder with an unknown owner address is 3 years under 717.1035 (not 5); the PA commissions rule is 1301.10(2) (not 1301.5); PA, FL and TX VDA descriptions replaced with the treasury pages' own terms. POSITIONS ADOPTED 10/6/2026: Texas applies the 3-year rule (no court decision or Comptroller ruling specifically on broker-to-agent commissions was found; the position rests on the statutory definitions and the Comptroller's MS02 table); the Philly and TUR forfeiture clauses are not relied on against an escheat claim. STILL OPEN for counsel's confirmation: (1) deposit date is a proxy for the payable date; (2) Missouri and DC not researched (no holder formed there, DC balance $0); (3) Texas VDA eligibility for an entity that has filed before is not stated on the Comptroller pages - ask when requesting.</t>
   </si>
   <si>
     <t xml:space="preserve">Counsel / unclaimed-property advisor.</t>
@@ -2114,7 +2138,7 @@
     <t xml:space="preserve">Verification status</t>
   </si>
   <si>
-    <t xml:space="preserve">Likely test for independent-contractor commissions (SHORT/LONG)</t>
+    <t xml:space="preserve">Adopted test for independent-contractor commissions (SHORT/LONG)</t>
   </si>
   <si>
     <t xml:space="preserve">Why</t>
@@ -2150,7 +2174,7 @@
     <t xml:space="preserve">LONG</t>
   </si>
   <si>
-    <t xml:space="preserve">Agents are independent contractors (confirmed by user). 72.1015 reaches only 'wages' as defined in Labor Code 61.001(7): compensation owed by an employer to an employee; 61.001(3)(B) excludes independent contractors. The Comptroller's own property-code table (Pub. 96-478, rev. March 2026) puts MS02 'Commissions' at 3 years and MS01 wages at 1 year. The 3-year general rule (72.101) is therefore the test. Verified from the statute and Comptroller text; counsel should confirm only that the agents' contractor status holds (the ICAs and the user say it does).</t>
+    <t xml:space="preserve">Agents are independent contractors (confirmed by user). 72.1015 reaches only 'wages' as defined in Labor Code 61.001(7): compensation owed by an employer to an employee; 61.001(3)(B) excludes independent contractors. The Comptroller's own property-code table (Pub. 96-478, rev. March 2026) puts MS02 'Commissions' at 3 years and MS01 wages at 1 year. The 3-year general rule (72.101) is the test. ADOPTED by management on 10/6/2026 after the statute and Comptroller text were verified; the 1-year wage rule is not applied.</t>
   </si>
   <si>
     <t xml:space="preserve">https://statutes.capitol.texas.gov/Docs/PR/htm/PR.72.htm ; https://statutes.capitol.texas.gov/Docs/PR/htm/PR.74.htm ; https://statutes.capitol.texas.gov/Docs/LA/htm/LA.61.htm ; https://www.claimittexas.gov/docs/96-478.pdf ; https://www.claimittexas.gov/app/holder-deadlines ; https://www.claimittexas.gov/app/disclosure-program ; https://www.comptroller.texas.gov/taxes/publications/96-576.php</t>
@@ -2318,7 +2342,7 @@
     <t xml:space="preserve">Priority rules (Texas v. New Jersey, 379 U.S. 674 (1965)): (1) the state of the owner's last-known address on the holder's books; (2) if no address, the holder's state of incorporation/formation. The user confirmed that for many older checks the agent is unknown: those items fall under rule (2) and go to the state where each LLC was formed. Per the Entity Management Database that is TEXAS for URE Dallas, URE Houston, Quick Close Properties (TUR), URE Chicago and URE Philadelphia (the last two are Texas LLCs registered as foreign entities in IL and PA), FLORIDA for RaySon Partners d/b/a URE Gallery and ALABAMA for Leading Edge Realty. Not the office's state, and not Kansas City. Private retention of amounts owed to others ('private escheat') is not permitted by any state; an unknown owner does not make the money the company's.</t>
   </si>
   <si>
-    <t xml:space="preserve">Blue = hardcoded inputs you can change. All dormancy periods are expressed in years and are applied from the DEPOSIT DATE in the cash-requirements workbook as a proxy for the date the amount became payable - the true trigger is when the agent's share became payable, which may be earlier (closing date) or later.</t>
+    <t xml:space="preserve">Blue = hardcoded inputs you can change. Tests in col M were adopted by management on 10/6/2026 after verification (Texas: 3-year rule). All dormancy periods are expressed in years and are applied from the DEPOSIT DATE in the cash-requirements workbook as a proxy for the date the amount became payable - the true trigger is when the agent's share became payable, which may be earlier (closing date) or later.</t>
   </si>
 </sst>
 </file>
@@ -22541,7 +22565,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
@@ -22833,6 +22857,48 @@
       </c>
       <c r="D22" s="15" t="s">
         <v>551</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="B23" s="27" t="s">
+        <v>552</v>
+      </c>
+      <c r="C23" s="15" t="s">
+        <v>553</v>
+      </c>
+      <c r="D23" s="15" t="s">
+        <v>551</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="11" t="n">
+        <v>21</v>
+      </c>
+      <c r="B24" s="27" t="s">
+        <v>554</v>
+      </c>
+      <c r="C24" s="15" t="s">
+        <v>555</v>
+      </c>
+      <c r="D24" s="15" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="11" t="n">
+        <v>22</v>
+      </c>
+      <c r="B25" s="27" t="s">
+        <v>557</v>
+      </c>
+      <c r="C25" s="15" t="s">
+        <v>558</v>
+      </c>
+      <c r="D25" s="15" t="s">
+        <v>559</v>
       </c>
     </row>
   </sheetData>
@@ -22864,12 +22930,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>552</v>
+        <v>560</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>553</v>
+        <v>561</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -22882,19 +22948,19 @@
         <v>8</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>554</v>
+        <v>562</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>555</v>
+        <v>563</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>556</v>
+        <v>564</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>557</v>
+        <v>565</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>558</v>
+        <v>566</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22902,19 +22968,19 @@
         <v>37</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>559</v>
+        <v>567</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>560</v>
+        <v>568</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>561</v>
+        <v>569</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>562</v>
+        <v>570</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>563</v>
+        <v>571</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22923,16 +22989,16 @@
       </c>
       <c r="B6" s="15"/>
       <c r="C6" s="15" t="s">
-        <v>564</v>
+        <v>572</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>565</v>
+        <v>573</v>
       </c>
       <c r="E6" s="15" t="s">
-        <v>566</v>
+        <v>574</v>
       </c>
       <c r="F6" s="15" t="s">
-        <v>567</v>
+        <v>575</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22941,16 +23007,16 @@
       </c>
       <c r="B7" s="15"/>
       <c r="C7" s="15" t="s">
-        <v>564</v>
+        <v>572</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>568</v>
+        <v>576</v>
       </c>
       <c r="E7" s="15" t="s">
-        <v>569</v>
+        <v>577</v>
       </c>
       <c r="F7" s="15" t="s">
-        <v>570</v>
+        <v>578</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22959,16 +23025,16 @@
       </c>
       <c r="B8" s="15"/>
       <c r="C8" s="15" t="s">
-        <v>564</v>
+        <v>572</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>571</v>
+        <v>579</v>
       </c>
       <c r="E8" s="15" t="s">
-        <v>572</v>
+        <v>580</v>
       </c>
       <c r="F8" s="15" t="s">
-        <v>573</v>
+        <v>581</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22977,16 +23043,16 @@
       </c>
       <c r="B9" s="15"/>
       <c r="C9" s="15" t="s">
-        <v>564</v>
+        <v>572</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>574</v>
+        <v>582</v>
       </c>
       <c r="E9" s="15" t="s">
-        <v>575</v>
+        <v>583</v>
       </c>
       <c r="F9" s="15" t="s">
-        <v>576</v>
+        <v>584</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22994,19 +23060,19 @@
         <v>44</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>577</v>
+        <v>585</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>578</v>
+        <v>586</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>579</v>
+        <v>587</v>
       </c>
       <c r="E10" s="15" t="s">
-        <v>580</v>
+        <v>588</v>
       </c>
       <c r="F10" s="15" t="s">
-        <v>581</v>
+        <v>589</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23015,16 +23081,16 @@
       </c>
       <c r="B11" s="15"/>
       <c r="C11" s="15" t="s">
-        <v>564</v>
+        <v>572</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>582</v>
+        <v>590</v>
       </c>
       <c r="E11" s="15" t="s">
-        <v>583</v>
+        <v>591</v>
       </c>
       <c r="F11" s="15" t="s">
-        <v>584</v>
+        <v>592</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23032,19 +23098,19 @@
         <v>40</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>585</v>
+        <v>593</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>586</v>
+        <v>594</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>587</v>
+        <v>595</v>
       </c>
       <c r="E12" s="15" t="s">
-        <v>588</v>
+        <v>596</v>
       </c>
       <c r="F12" s="15" t="s">
-        <v>589</v>
+        <v>597</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23053,16 +23119,16 @@
       </c>
       <c r="B13" s="15"/>
       <c r="C13" s="15" t="s">
-        <v>564</v>
+        <v>572</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>590</v>
+        <v>598</v>
       </c>
       <c r="E13" s="15" t="s">
-        <v>591</v>
+        <v>599</v>
       </c>
       <c r="F13" s="15" t="s">
-        <v>592</v>
+        <v>600</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23071,16 +23137,16 @@
       </c>
       <c r="B14" s="15"/>
       <c r="C14" s="15" t="s">
-        <v>564</v>
+        <v>572</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>593</v>
+        <v>601</v>
       </c>
       <c r="E14" s="15" t="s">
-        <v>594</v>
+        <v>602</v>
       </c>
       <c r="F14" s="15" t="s">
-        <v>595</v>
+        <v>603</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23089,16 +23155,16 @@
       </c>
       <c r="B15" s="15"/>
       <c r="C15" s="15" t="s">
-        <v>564</v>
+        <v>572</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>596</v>
+        <v>604</v>
       </c>
       <c r="E15" s="15" t="s">
-        <v>597</v>
+        <v>605</v>
       </c>
       <c r="F15" s="15" t="s">
-        <v>598</v>
+        <v>606</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23106,19 +23172,19 @@
         <v>42</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>599</v>
+        <v>607</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>600</v>
+        <v>608</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>601</v>
+        <v>609</v>
       </c>
       <c r="E16" s="15" t="s">
-        <v>602</v>
+        <v>610</v>
       </c>
       <c r="F16" s="15" t="s">
-        <v>603</v>
+        <v>611</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23127,16 +23193,16 @@
       </c>
       <c r="B17" s="15"/>
       <c r="C17" s="15" t="s">
-        <v>564</v>
+        <v>572</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>604</v>
+        <v>612</v>
       </c>
       <c r="E17" s="15" t="s">
-        <v>605</v>
+        <v>613</v>
       </c>
       <c r="F17" s="15" t="s">
-        <v>606</v>
+        <v>614</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23145,16 +23211,16 @@
       </c>
       <c r="B18" s="15"/>
       <c r="C18" s="15" t="s">
-        <v>564</v>
+        <v>572</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>607</v>
+        <v>615</v>
       </c>
       <c r="E18" s="15" t="s">
-        <v>608</v>
+        <v>616</v>
       </c>
       <c r="F18" s="15" t="s">
-        <v>609</v>
+        <v>617</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23163,16 +23229,16 @@
       </c>
       <c r="B19" s="15"/>
       <c r="C19" s="15" t="s">
-        <v>564</v>
+        <v>572</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>610</v>
+        <v>618</v>
       </c>
       <c r="E19" s="15" t="s">
-        <v>611</v>
+        <v>619</v>
       </c>
       <c r="F19" s="15" t="s">
-        <v>612</v>
+        <v>620</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23181,16 +23247,16 @@
       </c>
       <c r="B20" s="15"/>
       <c r="C20" s="15" t="s">
-        <v>564</v>
+        <v>572</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>613</v>
+        <v>621</v>
       </c>
       <c r="E20" s="15" t="s">
-        <v>614</v>
+        <v>622</v>
       </c>
       <c r="F20" s="15" t="s">
-        <v>615</v>
+        <v>623</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23198,19 +23264,19 @@
         <v>47</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>616</v>
+        <v>624</v>
       </c>
       <c r="C21" s="15" t="s">
-        <v>617</v>
+        <v>625</v>
       </c>
       <c r="D21" s="15" t="s">
-        <v>618</v>
+        <v>626</v>
       </c>
       <c r="E21" s="15" t="s">
-        <v>619</v>
+        <v>627</v>
       </c>
       <c r="F21" s="15" t="s">
-        <v>620</v>
+        <v>628</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23219,16 +23285,16 @@
       </c>
       <c r="B22" s="15"/>
       <c r="C22" s="15" t="s">
-        <v>564</v>
+        <v>572</v>
       </c>
       <c r="D22" s="15" t="s">
-        <v>621</v>
+        <v>629</v>
       </c>
       <c r="E22" s="15" t="s">
-        <v>622</v>
+        <v>630</v>
       </c>
       <c r="F22" s="15" t="s">
-        <v>623</v>
+        <v>631</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23237,16 +23303,16 @@
       </c>
       <c r="B23" s="15"/>
       <c r="C23" s="15" t="s">
-        <v>564</v>
+        <v>572</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>624</v>
+        <v>632</v>
       </c>
       <c r="E23" s="15" t="s">
-        <v>625</v>
+        <v>633</v>
       </c>
       <c r="F23" s="15" t="s">
-        <v>626</v>
+        <v>634</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23255,16 +23321,16 @@
       </c>
       <c r="B24" s="15"/>
       <c r="C24" s="15" t="s">
-        <v>564</v>
+        <v>572</v>
       </c>
       <c r="D24" s="15" t="s">
-        <v>627</v>
+        <v>635</v>
       </c>
       <c r="E24" s="15" t="s">
-        <v>628</v>
+        <v>636</v>
       </c>
       <c r="F24" s="15" t="s">
-        <v>629</v>
+        <v>637</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23273,56 +23339,56 @@
       </c>
       <c r="B25" s="15"/>
       <c r="C25" s="15" t="s">
-        <v>564</v>
+        <v>572</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>630</v>
+        <v>638</v>
       </c>
       <c r="E25" s="15" t="s">
-        <v>631</v>
+        <v>639</v>
       </c>
       <c r="F25" s="15" t="s">
-        <v>632</v>
+        <v>640</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="27" t="s">
-        <v>633</v>
+        <v>641</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>634</v>
+        <v>642</v>
       </c>
       <c r="C26" s="15" t="s">
-        <v>635</v>
+        <v>643</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>636</v>
+        <v>644</v>
       </c>
       <c r="E26" s="15" t="s">
-        <v>637</v>
+        <v>645</v>
       </c>
       <c r="F26" s="15" t="s">
-        <v>638</v>
+        <v>646</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="27" t="s">
-        <v>633</v>
+        <v>641</v>
       </c>
       <c r="B27" s="15" t="s">
-        <v>634</v>
+        <v>642</v>
       </c>
       <c r="C27" s="15" t="s">
-        <v>639</v>
+        <v>647</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>640</v>
+        <v>648</v>
       </c>
       <c r="E27" s="15" t="s">
-        <v>641</v>
+        <v>649</v>
       </c>
       <c r="F27" s="15" t="s">
-        <v>642</v>
+        <v>650</v>
       </c>
     </row>
   </sheetData>
@@ -23352,12 +23418,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>643</v>
+        <v>651</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>644</v>
+        <v>652</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -23371,7 +23437,7 @@
     </row>
     <row r="4" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>645</v>
+        <v>653</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -23385,7 +23451,7 @@
     </row>
     <row r="5" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>646</v>
+        <v>654</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -23399,7 +23465,7 @@
     </row>
     <row r="6" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>647</v>
+        <v>655</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -23413,7 +23479,7 @@
     </row>
     <row r="7" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>648</v>
+        <v>656</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -23427,7 +23493,7 @@
     </row>
     <row r="8" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>649</v>
+        <v>657</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -23441,7 +23507,7 @@
     </row>
     <row r="9" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>650</v>
+        <v>658</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -23455,7 +23521,7 @@
     </row>
     <row r="10" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>651</v>
+        <v>659</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -23469,7 +23535,7 @@
     </row>
     <row r="11" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>652</v>
+        <v>660</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -23483,7 +23549,7 @@
     </row>
     <row r="12" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>653</v>
+        <v>661</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -23497,7 +23563,7 @@
     </row>
     <row r="13" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>654</v>
+        <v>662</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -23558,12 +23624,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>655</v>
+        <v>663</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>656</v>
+        <v>664</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -23581,49 +23647,49 @@
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>657</v>
+        <v>665</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>658</v>
+        <v>666</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>23</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>659</v>
+        <v>667</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>24</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>660</v>
+        <v>668</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>661</v>
+        <v>669</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>662</v>
+        <v>670</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>663</v>
+        <v>671</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>664</v>
+        <v>672</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>665</v>
+        <v>673</v>
       </c>
       <c r="L4" s="6" t="s">
-        <v>666</v>
+        <v>674</v>
       </c>
       <c r="M4" s="6" t="s">
-        <v>667</v>
+        <v>675</v>
       </c>
       <c r="N4" s="6" t="s">
-        <v>668</v>
+        <v>676</v>
       </c>
       <c r="O4" s="6" t="s">
-        <v>669</v>
+        <v>677</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23631,46 +23697,46 @@
         <v>38</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>670</v>
+        <v>678</v>
       </c>
       <c r="C5" s="28" t="n">
         <v>1</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>671</v>
+        <v>679</v>
       </c>
       <c r="E5" s="28" t="n">
         <v>3</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>672</v>
+        <v>680</v>
       </c>
       <c r="G5" s="15" t="s">
-        <v>673</v>
+        <v>681</v>
       </c>
       <c r="H5" s="15" t="s">
-        <v>674</v>
+        <v>682</v>
       </c>
       <c r="I5" s="29" t="n">
         <v>46447</v>
       </c>
       <c r="J5" s="15" t="s">
-        <v>675</v>
+        <v>683</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>676</v>
+        <v>684</v>
       </c>
       <c r="L5" s="15" t="s">
-        <v>677</v>
+        <v>685</v>
       </c>
       <c r="M5" s="28" t="s">
-        <v>678</v>
+        <v>686</v>
       </c>
       <c r="N5" s="15" t="s">
-        <v>679</v>
+        <v>687</v>
       </c>
       <c r="O5" s="15" t="s">
-        <v>680</v>
+        <v>688</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23678,46 +23744,46 @@
         <v>45</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>681</v>
+        <v>689</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>1</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>682</v>
+        <v>690</v>
       </c>
       <c r="E6" s="28" t="n">
         <v>3</v>
       </c>
       <c r="F6" s="15" t="s">
-        <v>683</v>
+        <v>691</v>
       </c>
       <c r="G6" s="15" t="s">
-        <v>684</v>
+        <v>692</v>
       </c>
       <c r="H6" s="15" t="s">
-        <v>685</v>
+        <v>693</v>
       </c>
       <c r="I6" s="29" t="n">
         <v>46387</v>
       </c>
       <c r="J6" s="15" t="s">
-        <v>686</v>
+        <v>694</v>
       </c>
       <c r="K6" s="15" t="s">
-        <v>687</v>
+        <v>695</v>
       </c>
       <c r="L6" s="15" t="s">
-        <v>688</v>
+        <v>696</v>
       </c>
       <c r="M6" s="28" t="s">
-        <v>689</v>
+        <v>697</v>
       </c>
       <c r="N6" s="15" t="s">
-        <v>690</v>
+        <v>698</v>
       </c>
       <c r="O6" s="15" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23725,46 +23791,46 @@
         <v>48</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>692</v>
+        <v>700</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>2</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>693</v>
+        <v>701</v>
       </c>
       <c r="E7" s="28" t="n">
         <v>3</v>
       </c>
       <c r="F7" s="15" t="s">
-        <v>694</v>
+        <v>702</v>
       </c>
       <c r="G7" s="15" t="s">
-        <v>695</v>
+        <v>703</v>
       </c>
       <c r="H7" s="15" t="s">
-        <v>696</v>
+        <v>704</v>
       </c>
       <c r="I7" s="29" t="n">
         <v>46387</v>
       </c>
       <c r="J7" s="15" t="s">
+        <v>705</v>
+      </c>
+      <c r="K7" s="15" t="s">
+        <v>706</v>
+      </c>
+      <c r="L7" s="15" t="s">
+        <v>707</v>
+      </c>
+      <c r="M7" s="28" t="s">
         <v>697</v>
       </c>
-      <c r="K7" s="15" t="s">
-        <v>698</v>
-      </c>
-      <c r="L7" s="15" t="s">
-        <v>699</v>
-      </c>
-      <c r="M7" s="28" t="s">
-        <v>689</v>
-      </c>
       <c r="N7" s="15" t="s">
-        <v>700</v>
+        <v>708</v>
       </c>
       <c r="O7" s="15" t="s">
-        <v>701</v>
+        <v>709</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23772,46 +23838,46 @@
         <v>51</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>702</v>
+        <v>710</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>1</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>703</v>
+        <v>711</v>
       </c>
       <c r="E8" s="28" t="n">
         <v>3</v>
       </c>
       <c r="F8" s="15" t="s">
-        <v>704</v>
+        <v>712</v>
       </c>
       <c r="G8" s="15" t="s">
-        <v>705</v>
+        <v>713</v>
       </c>
       <c r="H8" s="15" t="s">
-        <v>706</v>
+        <v>714</v>
       </c>
       <c r="I8" s="29" t="n">
         <v>46387</v>
       </c>
       <c r="J8" s="15" t="s">
-        <v>707</v>
+        <v>715</v>
       </c>
       <c r="K8" s="15" t="s">
-        <v>708</v>
+        <v>716</v>
       </c>
       <c r="L8" s="15" t="s">
-        <v>709</v>
+        <v>717</v>
       </c>
       <c r="M8" s="28" t="s">
-        <v>678</v>
+        <v>686</v>
       </c>
       <c r="N8" s="15" t="s">
-        <v>710</v>
+        <v>718</v>
       </c>
       <c r="O8" s="15" t="s">
-        <v>711</v>
+        <v>719</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23819,93 +23885,93 @@
         <v>54</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>712</v>
+        <v>720</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>1</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="E9" s="28" t="n">
         <v>3</v>
       </c>
       <c r="F9" s="15" t="s">
-        <v>714</v>
+        <v>722</v>
       </c>
       <c r="G9" s="15" t="s">
-        <v>715</v>
+        <v>723</v>
       </c>
       <c r="H9" s="15" t="s">
-        <v>716</v>
+        <v>724</v>
       </c>
       <c r="I9" s="29" t="n">
         <v>46568</v>
       </c>
       <c r="J9" s="15" t="s">
-        <v>717</v>
+        <v>725</v>
       </c>
       <c r="K9" s="15" t="s">
-        <v>718</v>
+        <v>726</v>
       </c>
       <c r="L9" s="15" t="s">
-        <v>719</v>
+        <v>727</v>
       </c>
       <c r="M9" s="28" t="s">
-        <v>689</v>
+        <v>697</v>
       </c>
       <c r="N9" s="15" t="s">
-        <v>720</v>
+        <v>728</v>
       </c>
       <c r="O9" s="15" t="s">
-        <v>721</v>
+        <v>729</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>722</v>
+        <v>730</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>723</v>
+        <v>731</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>724</v>
+        <v>732</v>
       </c>
       <c r="E10" s="28" t="n">
         <v>5</v>
       </c>
       <c r="F10" s="15" t="s">
-        <v>725</v>
+        <v>733</v>
       </c>
       <c r="G10" s="15" t="s">
-        <v>726</v>
+        <v>734</v>
       </c>
       <c r="H10" s="15" t="s">
-        <v>716</v>
+        <v>724</v>
       </c>
       <c r="I10" s="29" t="n">
         <v>46568</v>
       </c>
       <c r="J10" s="15" t="s">
-        <v>727</v>
+        <v>735</v>
       </c>
       <c r="K10" s="15" t="s">
-        <v>728</v>
+        <v>736</v>
       </c>
       <c r="L10" s="15" t="s">
-        <v>729</v>
+        <v>737</v>
       </c>
       <c r="M10" s="28" t="s">
-        <v>678</v>
+        <v>686</v>
       </c>
       <c r="N10" s="15" t="s">
-        <v>730</v>
+        <v>738</v>
       </c>
       <c r="O10" s="15" t="s">
-        <v>731</v>
+        <v>739</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23913,15 +23979,15 @@
         <v>56</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>732</v>
+        <v>740</v>
       </c>
       <c r="C11" s="28"/>
       <c r="D11" s="15" t="s">
-        <v>733</v>
+        <v>741</v>
       </c>
       <c r="E11" s="28"/>
       <c r="F11" s="15" t="s">
-        <v>728</v>
+        <v>736</v>
       </c>
       <c r="G11" s="15"/>
       <c r="H11" s="15"/>
@@ -23929,17 +23995,17 @@
       <c r="J11" s="15"/>
       <c r="K11" s="15"/>
       <c r="L11" s="15" t="s">
-        <v>728</v>
+        <v>736</v>
       </c>
       <c r="M11" s="28"/>
       <c r="N11" s="15" t="s">
-        <v>728</v>
+        <v>736</v>
       </c>
       <c r="O11" s="15"/>
     </row>
     <row r="13" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>734</v>
+        <v>742</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -23958,7 +24024,7 @@
     </row>
     <row r="14" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>735</v>
+        <v>743</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>

</xml_diff>

<commit_message>
Move the review to twice a year and document the cost of a missed cutoff
Review cadence is now early December (as of Nov 30, ahead of the Dec 31 and
March 1 cutoffs) and early June (as of May 31, ahead of the June 30 cutoff
and the July 1 Texas remittance), owned by the Director of Financial
Reporting and Analysis. The SOP, one-pager, workbook Gaps tab and README
now carry the verified interest, penalty, waiver and enforcement-window
rules for each state when a cutoff is missed. Figures unchanged.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SVpE7ymJvQuwNuD1Yq5LvD
</commit_message>
<xml_diff>
--- a/accrued-commissions-analysis/Accrued_Commissions_Unclaimed_Property_Analysis.xlsx
+++ b/accrued-commissions-analysis/Accrued_Commissions_Unclaimed_Property_Analysis.xlsx
@@ -111,7 +111,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1693" uniqueCount="744">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1699" uniqueCount="749">
   <si>
     <t xml:space="preserve">Accrued Commissions - Unclaimed Property Exposure by Entity</t>
   </si>
@@ -293,7 +293,7 @@
     <t xml:space="preserve">How to read this</t>
   </si>
   <si>
-    <t xml:space="preserve">Classification (Detail col N) uses the fee amounts in rows 4-7 and the threshold in B8: an exact fee amount = company revenue, not unclaimed property. Decision 10/6/2026: fee checks are NOT moved to revenue en masse; they are recognized through the ordinary matching process and the year-end revenue true-up, and only an item being written off at a quarterly threshold review is booked to revenue at that time. At or under the threshold = likely fee, review. Memo-flagged = memo says not ours / unknown agent / duplicate / legal hold (owed back to the payer or needs resolution). Everything else = larger amount that likely includes an agent's commission split - this is the unclaimed-property population.</t>
+    <t xml:space="preserve">Classification (Detail col N) uses the fee amounts in rows 4-7 and the threshold in B8: an exact fee amount = company revenue, not unclaimed property. Decision 10/6/2026: fee checks are NOT moved to revenue en masse; they are recognized through the ordinary matching process and the year-end revenue true-up, and only an item being written off at a semi-annual threshold review is booked to revenue at that time. At or under the threshold = likely fee, review. Memo-flagged = memo says not ours / unknown agent / duplicate / legal hold (owed back to the payer or needs resolution). Everything else = larger amount that likely includes an agent's commission split - this is the unclaimed-property population.</t>
   </si>
   <si>
     <t xml:space="preserve">Columns R-S apply the dormancy tests to ALL unbooked items (upper bound). Columns T-W apply them only to the likely-commission and memo-flagged items. Even the T-W figures are upper bounds: within a larger check, only the agent's share (typically the check less the company's fee / split) is reportable; the company's share is revenue.</t>
@@ -1763,7 +1763,7 @@
     <t xml:space="preserve">DECISION: revenue timing for fee checks</t>
   </si>
   <si>
-    <t xml:space="preserve">Fee checks and confirmed small items are company revenue and are not unclaimed property, but they are NOT moved to revenue en masse. They stay in the accrued balance and are recognized when matched in the ordinary course and through the year-end revenue true-up, which already captures them. At a quarterly threshold review only an item that is being written off at that time is booked to revenue (decision 10/6/2026).</t>
+    <t xml:space="preserve">Fee checks and confirmed small items are company revenue and are not unclaimed property, but they are NOT moved to revenue en masse. They stay in the accrued balance and are recognized when matched in the ordinary course and through the year-end revenue true-up, which already captures them. At a semi-annual threshold review only an item that is being written off at that time is booked to revenue (decision 10/6/2026).</t>
   </si>
   <si>
     <t xml:space="preserve">Director of Financial Reporting and Analysis.</t>
@@ -1772,7 +1772,7 @@
     <t xml:space="preserve">DECISION: process owner</t>
   </si>
   <si>
-    <t xml:space="preserve">The quarterly threshold review and the annual state filings are owned by the Director of Financial Reporting and Analysis, with counsel; the CFO approves any VDA and any retention under an offset (decision 10/6/2026).</t>
+    <t xml:space="preserve">The semi-annual threshold review and the annual state filings are owned by the Director of Financial Reporting and Analysis, with counsel; the CFO approves any VDA and any retention under an offset (decision 10/6/2026).</t>
   </si>
   <si>
     <t xml:space="preserve">AFTER REMITTANCE: the agent later submits the file</t>
@@ -1782,6 +1782,21 @@
   </si>
   <si>
     <t xml:space="preserve">Director of Financial Reporting and Analysis / Accounting.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DECISION: review cadence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The threshold review runs twice a year, in early December (as of November 30, projected to the December 31 cutoffs for PA, IL and FL and the March 1 Texas cutoff) and early June (as of May 31, projected to the June 30 Alabama cutoff and the July 1 Texas remittance). The December review must finish before Pennsylvania's letter window closes on February 14; Texas letters go out by May 2 (decision 10/6/2026).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IF A CUTOFF IS MISSED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The item becomes past-due property and goes on the next report with its original dormancy date; nothing is forfeited. Verified consequences: Texas 10% interest a year from the original due date (74.705) plus a 5% penalty and a further 5% if more than 30 days late (74.706), waivable for a good-faith effort (74.707); Pennsylvania 12% interest (1301.24(b)) plus up to $1,000 a day (1301.24(c)), penalties waived for a good-faith, non-negligent holder (1301.25(c)); Florida $10 a day up to $500 for a late report (717.117(5)) and, if wilful, $500 a day up to $5,000 plus 25% of the unreported value (717.134), waived for good faith; Alabama $100 per business day up to $5,000, $500 a day up to $25,000 if wilful, waived for good faith (35-12-92); Illinois penalties and interest under the Act (not read in detail), forgone under the VDA. Enforcement windows run from a FILED report (TX 7 years, PA 15, IL and AL 10, FL 10 from the duty) and are tolled where nothing was reported, so unreported is worse than late.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Director of Financial Reporting and Analysis / counsel.</t>
   </si>
   <si>
     <t xml:space="preserve">VERIFIED 10/6/2026 - and what is still open</t>
@@ -22565,7 +22580,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
@@ -22898,7 +22913,35 @@
         <v>558</v>
       </c>
       <c r="D25" s="15" t="s">
+        <v>551</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="11" t="n">
+        <v>23</v>
+      </c>
+      <c r="B26" s="27" t="s">
         <v>559</v>
+      </c>
+      <c r="C26" s="15" t="s">
+        <v>560</v>
+      </c>
+      <c r="D26" s="15" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="11" t="n">
+        <v>24</v>
+      </c>
+      <c r="B27" s="27" t="s">
+        <v>562</v>
+      </c>
+      <c r="C27" s="15" t="s">
+        <v>563</v>
+      </c>
+      <c r="D27" s="15" t="s">
+        <v>564</v>
       </c>
     </row>
   </sheetData>
@@ -22930,12 +22973,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>560</v>
+        <v>565</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>561</v>
+        <v>566</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -22948,19 +22991,19 @@
         <v>8</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>562</v>
+        <v>567</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>563</v>
+        <v>568</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>564</v>
+        <v>569</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>565</v>
+        <v>570</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>566</v>
+        <v>571</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22968,19 +23011,19 @@
         <v>37</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>567</v>
+        <v>572</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>568</v>
+        <v>573</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>570</v>
+        <v>575</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>571</v>
+        <v>576</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22989,16 +23032,16 @@
       </c>
       <c r="B6" s="15"/>
       <c r="C6" s="15" t="s">
-        <v>572</v>
+        <v>577</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>573</v>
+        <v>578</v>
       </c>
       <c r="E6" s="15" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
       <c r="F6" s="15" t="s">
-        <v>575</v>
+        <v>580</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23007,16 +23050,16 @@
       </c>
       <c r="B7" s="15"/>
       <c r="C7" s="15" t="s">
-        <v>572</v>
+        <v>577</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>576</v>
+        <v>581</v>
       </c>
       <c r="E7" s="15" t="s">
-        <v>577</v>
+        <v>582</v>
       </c>
       <c r="F7" s="15" t="s">
-        <v>578</v>
+        <v>583</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23025,16 +23068,16 @@
       </c>
       <c r="B8" s="15"/>
       <c r="C8" s="15" t="s">
-        <v>572</v>
+        <v>577</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>579</v>
+        <v>584</v>
       </c>
       <c r="E8" s="15" t="s">
-        <v>580</v>
+        <v>585</v>
       </c>
       <c r="F8" s="15" t="s">
-        <v>581</v>
+        <v>586</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23043,16 +23086,16 @@
       </c>
       <c r="B9" s="15"/>
       <c r="C9" s="15" t="s">
-        <v>572</v>
+        <v>577</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>582</v>
+        <v>587</v>
       </c>
       <c r="E9" s="15" t="s">
-        <v>583</v>
+        <v>588</v>
       </c>
       <c r="F9" s="15" t="s">
-        <v>584</v>
+        <v>589</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23060,19 +23103,19 @@
         <v>44</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>585</v>
+        <v>590</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>586</v>
+        <v>591</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>587</v>
+        <v>592</v>
       </c>
       <c r="E10" s="15" t="s">
-        <v>588</v>
+        <v>593</v>
       </c>
       <c r="F10" s="15" t="s">
-        <v>589</v>
+        <v>594</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23081,16 +23124,16 @@
       </c>
       <c r="B11" s="15"/>
       <c r="C11" s="15" t="s">
-        <v>572</v>
+        <v>577</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>590</v>
+        <v>595</v>
       </c>
       <c r="E11" s="15" t="s">
-        <v>591</v>
+        <v>596</v>
       </c>
       <c r="F11" s="15" t="s">
-        <v>592</v>
+        <v>597</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23098,19 +23141,19 @@
         <v>40</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>593</v>
+        <v>598</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>594</v>
+        <v>599</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>595</v>
+        <v>600</v>
       </c>
       <c r="E12" s="15" t="s">
-        <v>596</v>
+        <v>601</v>
       </c>
       <c r="F12" s="15" t="s">
-        <v>597</v>
+        <v>602</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23119,16 +23162,16 @@
       </c>
       <c r="B13" s="15"/>
       <c r="C13" s="15" t="s">
-        <v>572</v>
+        <v>577</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>598</v>
+        <v>603</v>
       </c>
       <c r="E13" s="15" t="s">
-        <v>599</v>
+        <v>604</v>
       </c>
       <c r="F13" s="15" t="s">
-        <v>600</v>
+        <v>605</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23137,16 +23180,16 @@
       </c>
       <c r="B14" s="15"/>
       <c r="C14" s="15" t="s">
-        <v>572</v>
+        <v>577</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>601</v>
+        <v>606</v>
       </c>
       <c r="E14" s="15" t="s">
-        <v>602</v>
+        <v>607</v>
       </c>
       <c r="F14" s="15" t="s">
-        <v>603</v>
+        <v>608</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23155,16 +23198,16 @@
       </c>
       <c r="B15" s="15"/>
       <c r="C15" s="15" t="s">
-        <v>572</v>
+        <v>577</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>604</v>
+        <v>609</v>
       </c>
       <c r="E15" s="15" t="s">
-        <v>605</v>
+        <v>610</v>
       </c>
       <c r="F15" s="15" t="s">
-        <v>606</v>
+        <v>611</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23172,19 +23215,19 @@
         <v>42</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>607</v>
+        <v>612</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>608</v>
+        <v>613</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>609</v>
+        <v>614</v>
       </c>
       <c r="E16" s="15" t="s">
-        <v>610</v>
+        <v>615</v>
       </c>
       <c r="F16" s="15" t="s">
-        <v>611</v>
+        <v>616</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23193,16 +23236,16 @@
       </c>
       <c r="B17" s="15"/>
       <c r="C17" s="15" t="s">
-        <v>572</v>
+        <v>577</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>612</v>
+        <v>617</v>
       </c>
       <c r="E17" s="15" t="s">
-        <v>613</v>
+        <v>618</v>
       </c>
       <c r="F17" s="15" t="s">
-        <v>614</v>
+        <v>619</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23211,16 +23254,16 @@
       </c>
       <c r="B18" s="15"/>
       <c r="C18" s="15" t="s">
-        <v>572</v>
+        <v>577</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>615</v>
+        <v>620</v>
       </c>
       <c r="E18" s="15" t="s">
-        <v>616</v>
+        <v>621</v>
       </c>
       <c r="F18" s="15" t="s">
-        <v>617</v>
+        <v>622</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23229,16 +23272,16 @@
       </c>
       <c r="B19" s="15"/>
       <c r="C19" s="15" t="s">
-        <v>572</v>
+        <v>577</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>618</v>
+        <v>623</v>
       </c>
       <c r="E19" s="15" t="s">
-        <v>619</v>
+        <v>624</v>
       </c>
       <c r="F19" s="15" t="s">
-        <v>620</v>
+        <v>625</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23247,16 +23290,16 @@
       </c>
       <c r="B20" s="15"/>
       <c r="C20" s="15" t="s">
-        <v>572</v>
+        <v>577</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>621</v>
+        <v>626</v>
       </c>
       <c r="E20" s="15" t="s">
-        <v>622</v>
+        <v>627</v>
       </c>
       <c r="F20" s="15" t="s">
-        <v>623</v>
+        <v>628</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23264,19 +23307,19 @@
         <v>47</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>624</v>
+        <v>629</v>
       </c>
       <c r="C21" s="15" t="s">
-        <v>625</v>
+        <v>630</v>
       </c>
       <c r="D21" s="15" t="s">
-        <v>626</v>
+        <v>631</v>
       </c>
       <c r="E21" s="15" t="s">
-        <v>627</v>
+        <v>632</v>
       </c>
       <c r="F21" s="15" t="s">
-        <v>628</v>
+        <v>633</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23285,16 +23328,16 @@
       </c>
       <c r="B22" s="15"/>
       <c r="C22" s="15" t="s">
-        <v>572</v>
+        <v>577</v>
       </c>
       <c r="D22" s="15" t="s">
-        <v>629</v>
+        <v>634</v>
       </c>
       <c r="E22" s="15" t="s">
-        <v>630</v>
+        <v>635</v>
       </c>
       <c r="F22" s="15" t="s">
-        <v>631</v>
+        <v>636</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23303,16 +23346,16 @@
       </c>
       <c r="B23" s="15"/>
       <c r="C23" s="15" t="s">
-        <v>572</v>
+        <v>577</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>632</v>
+        <v>637</v>
       </c>
       <c r="E23" s="15" t="s">
-        <v>633</v>
+        <v>638</v>
       </c>
       <c r="F23" s="15" t="s">
-        <v>634</v>
+        <v>639</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23321,16 +23364,16 @@
       </c>
       <c r="B24" s="15"/>
       <c r="C24" s="15" t="s">
-        <v>572</v>
+        <v>577</v>
       </c>
       <c r="D24" s="15" t="s">
-        <v>635</v>
+        <v>640</v>
       </c>
       <c r="E24" s="15" t="s">
-        <v>636</v>
+        <v>641</v>
       </c>
       <c r="F24" s="15" t="s">
-        <v>637</v>
+        <v>642</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23339,56 +23382,56 @@
       </c>
       <c r="B25" s="15"/>
       <c r="C25" s="15" t="s">
-        <v>572</v>
+        <v>577</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>638</v>
+        <v>643</v>
       </c>
       <c r="E25" s="15" t="s">
-        <v>639</v>
+        <v>644</v>
       </c>
       <c r="F25" s="15" t="s">
-        <v>640</v>
+        <v>645</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="27" t="s">
-        <v>641</v>
+        <v>646</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>642</v>
+        <v>647</v>
       </c>
       <c r="C26" s="15" t="s">
-        <v>643</v>
+        <v>648</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>644</v>
+        <v>649</v>
       </c>
       <c r="E26" s="15" t="s">
-        <v>645</v>
+        <v>650</v>
       </c>
       <c r="F26" s="15" t="s">
-        <v>646</v>
+        <v>651</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="27" t="s">
-        <v>641</v>
+        <v>646</v>
       </c>
       <c r="B27" s="15" t="s">
-        <v>642</v>
+        <v>647</v>
       </c>
       <c r="C27" s="15" t="s">
-        <v>647</v>
+        <v>652</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>648</v>
+        <v>653</v>
       </c>
       <c r="E27" s="15" t="s">
-        <v>649</v>
+        <v>654</v>
       </c>
       <c r="F27" s="15" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
     </row>
   </sheetData>
@@ -23418,12 +23461,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>651</v>
+        <v>656</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>652</v>
+        <v>657</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -23437,7 +23480,7 @@
     </row>
     <row r="4" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>653</v>
+        <v>658</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -23451,7 +23494,7 @@
     </row>
     <row r="5" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>654</v>
+        <v>659</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -23465,7 +23508,7 @@
     </row>
     <row r="6" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>655</v>
+        <v>660</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -23479,7 +23522,7 @@
     </row>
     <row r="7" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>656</v>
+        <v>661</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -23493,7 +23536,7 @@
     </row>
     <row r="8" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>657</v>
+        <v>662</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -23507,7 +23550,7 @@
     </row>
     <row r="9" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>658</v>
+        <v>663</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -23521,7 +23564,7 @@
     </row>
     <row r="10" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>659</v>
+        <v>664</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -23535,7 +23578,7 @@
     </row>
     <row r="11" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>660</v>
+        <v>665</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -23549,7 +23592,7 @@
     </row>
     <row r="12" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>661</v>
+        <v>666</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -23563,7 +23606,7 @@
     </row>
     <row r="13" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>662</v>
+        <v>667</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -23624,12 +23667,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>663</v>
+        <v>668</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>664</v>
+        <v>669</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -23647,49 +23690,49 @@
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>665</v>
+        <v>670</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>666</v>
+        <v>671</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>23</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>667</v>
+        <v>672</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>24</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>668</v>
+        <v>673</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>669</v>
+        <v>674</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>670</v>
+        <v>675</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>671</v>
+        <v>676</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>672</v>
+        <v>677</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>673</v>
+        <v>678</v>
       </c>
       <c r="L4" s="6" t="s">
-        <v>674</v>
+        <v>679</v>
       </c>
       <c r="M4" s="6" t="s">
-        <v>675</v>
+        <v>680</v>
       </c>
       <c r="N4" s="6" t="s">
-        <v>676</v>
+        <v>681</v>
       </c>
       <c r="O4" s="6" t="s">
-        <v>677</v>
+        <v>682</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23697,46 +23740,46 @@
         <v>38</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>678</v>
+        <v>683</v>
       </c>
       <c r="C5" s="28" t="n">
         <v>1</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>679</v>
+        <v>684</v>
       </c>
       <c r="E5" s="28" t="n">
         <v>3</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>680</v>
+        <v>685</v>
       </c>
       <c r="G5" s="15" t="s">
-        <v>681</v>
+        <v>686</v>
       </c>
       <c r="H5" s="15" t="s">
-        <v>682</v>
+        <v>687</v>
       </c>
       <c r="I5" s="29" t="n">
         <v>46447</v>
       </c>
       <c r="J5" s="15" t="s">
-        <v>683</v>
+        <v>688</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>684</v>
+        <v>689</v>
       </c>
       <c r="L5" s="15" t="s">
-        <v>685</v>
+        <v>690</v>
       </c>
       <c r="M5" s="28" t="s">
-        <v>686</v>
+        <v>691</v>
       </c>
       <c r="N5" s="15" t="s">
-        <v>687</v>
+        <v>692</v>
       </c>
       <c r="O5" s="15" t="s">
-        <v>688</v>
+        <v>693</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23744,46 +23787,46 @@
         <v>45</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>689</v>
+        <v>694</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>1</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>690</v>
+        <v>695</v>
       </c>
       <c r="E6" s="28" t="n">
         <v>3</v>
       </c>
       <c r="F6" s="15" t="s">
-        <v>691</v>
+        <v>696</v>
       </c>
       <c r="G6" s="15" t="s">
-        <v>692</v>
+        <v>697</v>
       </c>
       <c r="H6" s="15" t="s">
-        <v>693</v>
+        <v>698</v>
       </c>
       <c r="I6" s="29" t="n">
         <v>46387</v>
       </c>
       <c r="J6" s="15" t="s">
-        <v>694</v>
+        <v>699</v>
       </c>
       <c r="K6" s="15" t="s">
-        <v>695</v>
+        <v>700</v>
       </c>
       <c r="L6" s="15" t="s">
-        <v>696</v>
+        <v>701</v>
       </c>
       <c r="M6" s="28" t="s">
-        <v>697</v>
+        <v>702</v>
       </c>
       <c r="N6" s="15" t="s">
-        <v>698</v>
+        <v>703</v>
       </c>
       <c r="O6" s="15" t="s">
-        <v>699</v>
+        <v>704</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23791,46 +23834,46 @@
         <v>48</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>700</v>
+        <v>705</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>2</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>701</v>
+        <v>706</v>
       </c>
       <c r="E7" s="28" t="n">
         <v>3</v>
       </c>
       <c r="F7" s="15" t="s">
-        <v>702</v>
+        <v>707</v>
       </c>
       <c r="G7" s="15" t="s">
-        <v>703</v>
+        <v>708</v>
       </c>
       <c r="H7" s="15" t="s">
-        <v>704</v>
+        <v>709</v>
       </c>
       <c r="I7" s="29" t="n">
         <v>46387</v>
       </c>
       <c r="J7" s="15" t="s">
-        <v>705</v>
+        <v>710</v>
       </c>
       <c r="K7" s="15" t="s">
-        <v>706</v>
+        <v>711</v>
       </c>
       <c r="L7" s="15" t="s">
-        <v>707</v>
+        <v>712</v>
       </c>
       <c r="M7" s="28" t="s">
-        <v>697</v>
+        <v>702</v>
       </c>
       <c r="N7" s="15" t="s">
-        <v>708</v>
+        <v>713</v>
       </c>
       <c r="O7" s="15" t="s">
-        <v>709</v>
+        <v>714</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23838,46 +23881,46 @@
         <v>51</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>710</v>
+        <v>715</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>1</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>711</v>
+        <v>716</v>
       </c>
       <c r="E8" s="28" t="n">
         <v>3</v>
       </c>
       <c r="F8" s="15" t="s">
-        <v>712</v>
+        <v>717</v>
       </c>
       <c r="G8" s="15" t="s">
-        <v>713</v>
+        <v>718</v>
       </c>
       <c r="H8" s="15" t="s">
-        <v>714</v>
+        <v>719</v>
       </c>
       <c r="I8" s="29" t="n">
         <v>46387</v>
       </c>
       <c r="J8" s="15" t="s">
-        <v>715</v>
+        <v>720</v>
       </c>
       <c r="K8" s="15" t="s">
-        <v>716</v>
+        <v>721</v>
       </c>
       <c r="L8" s="15" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
       <c r="M8" s="28" t="s">
-        <v>686</v>
+        <v>691</v>
       </c>
       <c r="N8" s="15" t="s">
-        <v>718</v>
+        <v>723</v>
       </c>
       <c r="O8" s="15" t="s">
-        <v>719</v>
+        <v>724</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23885,93 +23928,93 @@
         <v>54</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>720</v>
+        <v>725</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>1</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>721</v>
+        <v>726</v>
       </c>
       <c r="E9" s="28" t="n">
         <v>3</v>
       </c>
       <c r="F9" s="15" t="s">
-        <v>722</v>
+        <v>727</v>
       </c>
       <c r="G9" s="15" t="s">
-        <v>723</v>
+        <v>728</v>
       </c>
       <c r="H9" s="15" t="s">
-        <v>724</v>
+        <v>729</v>
       </c>
       <c r="I9" s="29" t="n">
         <v>46568</v>
       </c>
       <c r="J9" s="15" t="s">
-        <v>725</v>
+        <v>730</v>
       </c>
       <c r="K9" s="15" t="s">
-        <v>726</v>
+        <v>731</v>
       </c>
       <c r="L9" s="15" t="s">
-        <v>727</v>
+        <v>732</v>
       </c>
       <c r="M9" s="28" t="s">
-        <v>697</v>
+        <v>702</v>
       </c>
       <c r="N9" s="15" t="s">
-        <v>728</v>
+        <v>733</v>
       </c>
       <c r="O9" s="15" t="s">
-        <v>729</v>
+        <v>734</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>730</v>
+        <v>735</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>731</v>
+        <v>736</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>732</v>
+        <v>737</v>
       </c>
       <c r="E10" s="28" t="n">
         <v>5</v>
       </c>
       <c r="F10" s="15" t="s">
-        <v>733</v>
+        <v>738</v>
       </c>
       <c r="G10" s="15" t="s">
-        <v>734</v>
+        <v>739</v>
       </c>
       <c r="H10" s="15" t="s">
-        <v>724</v>
+        <v>729</v>
       </c>
       <c r="I10" s="29" t="n">
         <v>46568</v>
       </c>
       <c r="J10" s="15" t="s">
-        <v>735</v>
+        <v>740</v>
       </c>
       <c r="K10" s="15" t="s">
-        <v>736</v>
+        <v>741</v>
       </c>
       <c r="L10" s="15" t="s">
-        <v>737</v>
+        <v>742</v>
       </c>
       <c r="M10" s="28" t="s">
-        <v>686</v>
+        <v>691</v>
       </c>
       <c r="N10" s="15" t="s">
-        <v>738</v>
+        <v>743</v>
       </c>
       <c r="O10" s="15" t="s">
-        <v>739</v>
+        <v>744</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23979,15 +24022,15 @@
         <v>56</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>740</v>
+        <v>745</v>
       </c>
       <c r="C11" s="28"/>
       <c r="D11" s="15" t="s">
-        <v>741</v>
+        <v>746</v>
       </c>
       <c r="E11" s="28"/>
       <c r="F11" s="15" t="s">
-        <v>736</v>
+        <v>741</v>
       </c>
       <c r="G11" s="15"/>
       <c r="H11" s="15"/>
@@ -23995,17 +24038,17 @@
       <c r="J11" s="15"/>
       <c r="K11" s="15"/>
       <c r="L11" s="15" t="s">
-        <v>736</v>
+        <v>741</v>
       </c>
       <c r="M11" s="28"/>
       <c r="N11" s="15" t="s">
-        <v>736</v>
+        <v>741</v>
       </c>
       <c r="O11" s="15"/>
     </row>
     <row r="13" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>742</v>
+        <v>747</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -24024,7 +24067,7 @@
     </row>
     <row r="14" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>743</v>
+        <v>748</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>

</xml_diff>

<commit_message>
Move to one annual cycle: December review, January letters, statutory filing dates
A single review in early December (as of Nov 30) is projected to every
state cutoff; one batch of due-diligence letters goes out Jan 1 to Feb 14,
inside every state's window; reports are prepared together and submitted on
the statutory dates (PA Apr 15, IL and FL May 1, TX Jul 1, AL Nov 1). The
June review is dropped. SOP, one-pager, rollout note, workbook notes,
README and handoff updated. Figures unchanged.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SVpE7ymJvQuwNuD1Yq5LvD
</commit_message>
<xml_diff>
--- a/accrued-commissions-analysis/Accrued_Commissions_Unclaimed_Property_Analysis.xlsx
+++ b/accrued-commissions-analysis/Accrued_Commissions_Unclaimed_Property_Analysis.xlsx
@@ -293,7 +293,7 @@
     <t xml:space="preserve">How to read this</t>
   </si>
   <si>
-    <t xml:space="preserve">Classification (Detail col N) uses the fee amounts in rows 4-7 and the threshold in B8: an exact fee amount = company revenue, not unclaimed property. Decision 10/6/2026: fee checks are NOT moved to revenue en masse; they are recognized through the ordinary matching process and the year-end revenue true-up, and only an item being written off at a semi-annual threshold review is booked to revenue at that time. At or under the threshold = likely fee, review. Memo-flagged = memo says not ours / unknown agent / duplicate / legal hold (owed back to the payer or needs resolution). Everything else = larger amount that likely includes an agent's commission split - this is the unclaimed-property population.</t>
+    <t xml:space="preserve">Classification (Detail col N) uses the fee amounts in rows 4-7 and the threshold in B8: an exact fee amount = company revenue, not unclaimed property. Decision 10/6/2026: fee checks are NOT moved to revenue en masse; they are recognized through the ordinary matching process and the year-end revenue true-up, and only an item being written off at the annual threshold review is booked to revenue at that time. At or under the threshold = likely fee, review. Memo-flagged = memo says not ours / unknown agent / duplicate / legal hold (owed back to the payer or needs resolution). Everything else = larger amount that likely includes an agent's commission split - this is the unclaimed-property population.</t>
   </si>
   <si>
     <t xml:space="preserve">Columns R-S apply the dormancy tests to ALL unbooked items (upper bound). Columns T-W apply them only to the likely-commission and memo-flagged items. Even the T-W figures are upper bounds: within a larger check, only the agent's share (typically the check less the company's fee / split) is reportable; the company's share is revenue.</t>
@@ -1763,7 +1763,7 @@
     <t xml:space="preserve">DECISION: revenue timing for fee checks</t>
   </si>
   <si>
-    <t xml:space="preserve">Fee checks and confirmed small items are company revenue and are not unclaimed property, but they are NOT moved to revenue en masse. They stay in the accrued balance and are recognized when matched in the ordinary course and through the year-end revenue true-up, which already captures them. At a semi-annual threshold review only an item that is being written off at that time is booked to revenue (decision 10/6/2026).</t>
+    <t xml:space="preserve">Fee checks and confirmed small items are company revenue and are not unclaimed property, but they are NOT moved to revenue en masse. They stay in the accrued balance and are recognized when matched in the ordinary course and through the year-end revenue true-up, which already captures them. At the annual threshold review only an item that is being written off at that time is booked to revenue (decision 10/6/2026).</t>
   </si>
   <si>
     <t xml:space="preserve">Director of Financial Reporting and Analysis.</t>
@@ -1772,7 +1772,7 @@
     <t xml:space="preserve">DECISION: process owner</t>
   </si>
   <si>
-    <t xml:space="preserve">The semi-annual threshold review and the annual state filings are owned by the Director of Financial Reporting and Analysis, with counsel; the CFO approves any VDA and any retention under an offset (decision 10/6/2026).</t>
+    <t xml:space="preserve">The annual threshold review and the state filings are owned by the Director of Financial Reporting and Analysis, with counsel; the CFO approves any VDA and any retention under an offset (decision 10/6/2026).</t>
   </si>
   <si>
     <t xml:space="preserve">AFTER REMITTANCE: the agent later submits the file</t>
@@ -1784,10 +1784,10 @@
     <t xml:space="preserve">Director of Financial Reporting and Analysis / Accounting.</t>
   </si>
   <si>
-    <t xml:space="preserve">DECISION: review cadence</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The threshold review runs twice a year, in early December (as of November 30, projected to the December 31 cutoffs for PA, IL and FL and the March 1 Texas cutoff) and early June (as of May 31, projected to the June 30 Alabama cutoff and the July 1 Texas remittance). The December review must finish before Pennsylvania's letter window closes on February 14; Texas letters go out by May 2 (decision 10/6/2026).</t>
+    <t xml:space="preserve">DECISION: review cadence - one annual cycle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The threshold review runs once a year, in early December (as of November 30), projected forward to every state cutoff: December 31 for PA, IL and FL; March 1 for Texas; June 30 for Alabama. One batch of due-diligence letters goes out between January 1 and February 14, which is inside the PA (Dec 16 - Feb 14) and FL (Jan 1 - Mar 2) windows and earlier than IL, TX and AL require. Reports are prepared in the same cycle and submitted on each state's statutory date: PA April 15, IL and FL May 1, TX July 1, AL November 1. The review must finish before February 14. Not verified: whether TX and IL accept a report filed months early and whether AL accepts early remittance (decision 10/6/2026).</t>
   </si>
   <si>
     <t xml:space="preserve">IF A CUTOFF IS MISSED</t>

</xml_diff>

<commit_message>
Align every document with the adopted decisions
Workbook notes, ICA Terms rows, README, handoff and the archived prompt no
longer describe the Texas period or the forfeiture clauses as open counsel
questions; they state the 10/6/2026 positions. SOP CFO role line updated.
The previous commit's one-pager is at 8.5-point text, not 9. Figures
unchanged; Summary ties to 226,764.46.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SVpE7ymJvQuwNuD1Yq5LvD
</commit_message>
<xml_diff>
--- a/accrued-commissions-analysis/Accrued_Commissions_Unclaimed_Property_Analysis.xlsx
+++ b/accrued-commissions-analysis/Accrued_Commissions_Unclaimed_Property_Analysis.xlsx
@@ -299,7 +299,7 @@
     <t xml:space="preserve">Columns R-S apply the dormancy tests to ALL unbooked items (upper bound). Columns T-W apply them only to the likely-commission and memo-flagged items. Even the T-W figures are upper bounds: within a larger check, only the agent's share (typically the check less the company's fee / split) is reportable; the company's share is revenue.</t>
   </si>
   <si>
-    <t xml:space="preserve">SHORT test = the state's period for wages / compensation for personal services. LONG test = the general catch-all period. Column X picks the likely test for each entity's default governing state now that agents are confirmed to be independent contractors (Texas and Florida: LONG; Illinois, Pennsylvania, Alabama: SHORT), and columns Y-Z apply it item by item, so an item whose owner state has been filled in uses its own state's test. See State Rules cols M-N for the basis. Management adopted these tests on 10/6/2026 after the statutes were verified; Texas applies the 3-year rule and the 1-year wage rule is not used.</t>
+    <t xml:space="preserve">SHORT test = the state's period for wages / compensation for personal services. LONG test = the general catch-all period. Column X applies the test management adopted on 10/6/2026 for each entity's default governing state, agents being independent contractors (Texas and Florida: LONG; Illinois, Pennsylvania, Alabama: SHORT), and columns Y-Z apply it item by item, so an item whose owner state has been filled in uses its own state's test. See State Rules cols M-N for the basis. Management adopted these tests on 10/6/2026 after the statutes were verified; Texas applies the 3-year rule and the 1-year wage rule is not used.</t>
   </si>
   <si>
     <t xml:space="preserve">Unknown agent = second priority rule. Per the Entity Management Database, URE Dallas, URE Houston, Quick Close Properties (TUR), URE Chicago and URE Philadelphia are all TEXAS LLCs; Gallery (RaySon Partners) is Florida; Leading Edge Realty is Alabama. Column B holds that formation state as each entity's DEFAULT governing state, so unknown-agent items at Chicago and Philly are tested under TEXAS rules (3-year general period for contractor commissions), not Illinois or Pennsylvania. When an agent's last-known address state is entered in Detail col U, that item switches to the address state's rules (first priority rule). Office state is shown in col AB for reference.</t>
@@ -308,7 +308,7 @@
     <t xml:space="preserve">Current-month accrued (column D) is all September/October 2026 deposits in normal matching workflow. It is included so the total ties to the cash-requirements Summary, but none of it is near any dormancy period.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nothing here is legal advice. Dormancy periods, report dates, due-diligence rules, VDA terms and anti-limitation provisions on the State Rules tab were verified against the statute text and state treasury pages on 10/6/2026 (URLs in the Sources column). They state the rules; applying them to independent-contractor commissions and to the ICA forfeiture clauses is a judgment for counsel to confirm before filing.</t>
+    <t xml:space="preserve">Nothing here is legal advice. Dormancy periods, report dates, due-diligence rules, VDA terms and anti-limitation provisions on the State Rules tab were verified against the statute text and state treasury pages on 10/6/2026 (URLs in the Sources column). Management adopted the Texas 3-year test and decided not to rely on the ICA forfeiture clauses on 10/6/2026; counsel confirms the positions before the first filing.</t>
   </si>
   <si>
     <t xml:space="preserve">Unbooked deposited checks - item detail (prior-month accrued commissions block of each entity tab)</t>
@@ -1670,10 +1670,10 @@
     <t xml:space="preserve">RESOLVED: agents are independent contractors</t>
   </si>
   <si>
-    <t xml:space="preserve">User confirmed 10/6/2026. Verified 10/6/2026 from the statute text: Texas' 1-year rule applies to 'wages' as defined in Labor Code 61.001, which excludes independent contractors, and the Comptroller's property-code table puts commissions (MS02) at 3 years, so the 3-year general rule is the Texas test. Illinois, Pennsylvania and Alabama each reach 'other compensation for personal services', so their shorter periods apply. Florida's wage rule is not shown to reach contractors, so 5 years is likely. Counsel should confirm each.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Confirm with counsel.</t>
+    <t xml:space="preserve">User confirmed 10/6/2026. Verified 10/6/2026 from the statute text: Texas' 1-year rule applies to 'wages' as defined in Labor Code 61.001, which excludes independent contractors, and the Comptroller's property-code table puts commissions (MS02) at 3 years, so the 3-year general rule is the Texas test. Illinois, Pennsylvania and Alabama each reach 'other compensation for personal services', so their shorter periods apply. Florida's wage rule does not reach contractors; a Florida holder with an unknown owner address uses 717.1035 (3 years), and 717.102 (5 years) where the owner has a Florida address. Positions adopted by management 10/6/2026; counsel confirms before the first filing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adopted 10/6/2026.</t>
   </si>
   <si>
     <t xml:space="preserve">RESOLVED: no prior write-offs</t>
@@ -1988,7 +1988,7 @@
     <t xml:space="preserve">1.K: an agent who collects a fee in their own name 'will forfeit any accrued but uncollected commissions'. 3.B: agent assigns commissions to TUR to secure indemnification. 5.F: breach of Section 5 (confidentiality / non-solicitation) means the agent 'shall lose all rights to any further commissions'. 8.C: amounts owed at or after termination may be deducted from commissions due.</t>
   </si>
   <si>
-    <t xml:space="preserve">Offset (8.C, 3.B) is a documented reduction. Forfeiture (1.K, 5.F) is a legal question: anti-limitation provisions in unclaimed property acts may override a contractual forfeiture. Do not rely on it without counsel and a documented breach.</t>
+    <t xml:space="preserve">Offset (8.C, 3.B) is a documented reduction. Forfeiture (1.K, 5.F) is not relied on against an escheat claim (decision 10/6/2026): Texas 74.308 disregards contract-based limits and 74.309 bars private escheat. It may be applied only to an item settled in the ordinary course before dormancy, with the breach documented.</t>
   </si>
   <si>
     <t xml:space="preserve">Policies item 6 Record Keeping</t>
@@ -2030,7 +2030,7 @@
     <t xml:space="preserve">Post-termination commissions disbursed per the plan in effect, 'conditioned on Contractor having any and all dues, fees and expenses owing to Broker paid in full.' Broker may 'hold and/or apply any commissions owing to Contractor' to secure obligations. On termination, executed contracts split 70/30. 'If the Contractor's license expires or goes inactive, anything that is currently under contract brokerage split will be fifty/fifty. Contractor will have 30 days to bring their license back to active status. If Contractor fails to bring license back to active status within the 30 days, brokerage will keep 100% of commission.'</t>
   </si>
   <si>
-    <t xml:space="preserve">Offset rights as elsewhere, plus an express 100% retention clause for lapsed licenses. Whether Pennsylvania unclaimed property law honors a contractual retention against an escheat claim is for counsel.</t>
+    <t xml:space="preserve">Offset rights as elsewhere, plus an express 100% retention clause for lapsed licenses. Decision 10/6/2026: not relied on against an escheat claim; the Pennsylvania act is silent on contract-based bars and most Philly items default to Texas, where 74.308-74.309 apply.</t>
   </si>
   <si>
     <t xml:space="preserve">Para. 31 Fines and Penalties</t>
@@ -2039,7 +2039,7 @@
     <t xml:space="preserve">'3. Any incomplete file(s) 30 days past closing will be paid at a 50/50 split. 4. Any incomplete file(s) 60 days past closing will be forfeited and grounds for termination.'</t>
   </si>
   <si>
-    <t xml:space="preserve">The most consequential clause for Philly's aged items: if a file was never completed, the ICA says the agent's share was forfeited at day 60 after closing. If counsel concludes Pennsylvania (or the agent's address state) honors this, those amounts are company revenue, not unclaimed property. Document the closing date and file status for each item before relying on it; anti-limitation provisions may override.</t>
+    <t xml:space="preserve">The most consequential clause for Philly's aged items: if a file was never completed, the ICA says the agent's share was forfeited at day 60 after closing. Decision 10/6/2026: the clause is not relied on against an escheat claim, so an aged Philly item is paid or reported at the agent's share whether or not the file was completed; the clause may be applied only to an item settled in the ordinary course before dormancy, with the day-60 file status documented.</t>
   </si>
   <si>
     <t xml:space="preserve">Para. 26 Contractor Information; Para. 28 Controlling Law; Para. 30 Paperless Pipeline</t>
@@ -2249,7 +2249,7 @@
     <t xml:space="preserve">Treasury Voluntary Disclosure Agreement (searchandclaimpa.gov/docs/PA_Voluntary_Disclosure_Agreement.pdf): Treasury waives penalties and interest under 1301.24 and 1301.25 for property reported within the agreement; the holder must be coming forward voluntarily, not be under audit or self-audit, and not have had voluntary compliance in the past 10 years; 10-year look-back; report within 90 days of execution; no report may be filed before Treasury's signed approval. Without a VDA: interest of 12% per year from when the report was due (1301.24(b)) and a penalty of up to $1,000 per day (1301.24(c)); the Treasurer may waive for good cause and must waive penalties where the holder acted in good faith and without negligence (1301.25(c)). The prior draft's statement that PA's program ended in 2010 referred to a one-time amnesty and is superseded.</t>
   </si>
   <si>
-    <t xml:space="preserve">VERIFIED on 10/6/2026 from the statute text as published by PA Treasury (PA_UCP_Law.pdf: 1301.6, 1301.10, 1301.10a, 1301.11, 1301.13, 1301.16, 1301.24, 1301.25 read), the Treasury Dormancy Matrix, the Holder Reporting Handbook, the Reporting Guidelines page and the VDA form. The General Assembly's own viewer for 1929 Act 176 Art. XIII.1 (palegis.us) returned only its page shell and its PDF link returned an error, so the Treasury reprint is the text relied on. ANTI-LIMITATION: 1301.16 - expiration of any period specified by STATUTE OR COURT ORDER during which the owner could sue the holder does not prevent custody or affect the duty to report; unlike TX, IL, FL and AL it does NOT mention periods set by contract, and the Act contains no private-escheat prohibition equivalent to Tex. Prop. Code 74.309. The Philly ICA 60-day forfeiture clause is therefore not answered by the Pennsylvania statute either way; it is a contract-law question for counsel. Most Philly items default to Texas, where 74.308 and 74.309 apply.</t>
+    <t xml:space="preserve">VERIFIED on 10/6/2026 from the statute text as published by PA Treasury (PA_UCP_Law.pdf: 1301.6, 1301.10, 1301.10a, 1301.11, 1301.13, 1301.16, 1301.24, 1301.25 read), the Treasury Dormancy Matrix, the Holder Reporting Handbook, the Reporting Guidelines page and the VDA form. The General Assembly's own viewer for 1929 Act 176 Art. XIII.1 (palegis.us) returned only its page shell and its PDF link returned an error, so the Treasury reprint is the text relied on. ANTI-LIMITATION: 1301.16 - expiration of any period specified by STATUTE OR COURT ORDER during which the owner could sue the holder does not prevent custody or affect the duty to report; unlike TX, IL, FL and AL it does NOT mention periods set by contract, and the Act contains no private-escheat prohibition equivalent to Tex. Prop. Code 74.309. The Philly ICA 60-day forfeiture clause is therefore not answered by the Pennsylvania statute either way; management decided on 10/6/2026 not to rely on it against an escheat claim. Most Philly items default to Texas, where 74.308 and 74.309 apply.</t>
   </si>
   <si>
     <t xml:space="preserve">1301.10(2) reaches 'wages or other compensation for personal services', and Treasury's handbook, matrix and VDA form all describe the 2-year exception as covering commissions. 3-year rule (1301.10(1)) is the fallback. Verified from the statute text.</t>

</xml_diff>